<commit_message>
Prokure: baja de Homero Ruiz (Continental) - fuera de Tanda 1, marcado en base, pendiente reemplazo
</commit_message>
<xml_diff>
--- a/GrowProkure/02-Investigacion/plasticos/Contactos_Foil_TID_Global.xlsx
+++ b/GrowProkure/02-Investigacion/plasticos/Contactos_Foil_TID_Global.xlsx
@@ -575,13 +575,13 @@
         </is>
       </c>
     </row>
+    <row r="3"/>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>TOTALES GLOBALES</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
@@ -630,7 +630,6 @@
           <t>BASE DE PROSPECCIÓN (Wiza+Apollo+ZoomInfo)</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
@@ -701,7 +700,6 @@
           <t>AGENDA PROPIA (iPhone, validada)</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
@@ -754,7 +752,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M66"/>
+  <dimension ref="A1:N66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -779,6 +777,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -2311,6 +2310,11 @@
       <c r="M27" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>BAJA 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -4724,6 +4728,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -6027,7 +6032,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M123"/>
+  <dimension ref="A1:N123"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -6052,6 +6057,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
@@ -7584,6 +7590,11 @@
       <c r="M27" s="8" t="inlineStr">
         <is>
           <t>Alta</t>
+        </is>
+      </c>
+      <c r="N27" t="inlineStr">
+        <is>
+          <t>BAJA 2026-07-15</t>
         </is>
       </c>
     </row>
@@ -13360,6 +13371,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>

</xml_diff>